<commit_message>
Summary personal untuk Mobile Promoters/PA/SPA, login mendarat di Summary, tombol CSV khusus admin, target Catur Agil Kurniawan
</commit_message>
<xml_diff>
--- a/Target.xlsx
+++ b/Target.xlsx
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1533" uniqueCount="333">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1538" uniqueCount="334">
   <si>
     <t>Store</t>
   </si>
@@ -462,6 +462,9 @@
   </si>
   <si>
     <t>Digiplus Jogja City Mall</t>
+  </si>
+  <si>
+    <t>Catur Agil Kurniawan</t>
   </si>
   <si>
     <t>Digiplus K Square Mall</t>
@@ -7615,7 +7618,9 @@
       <c r="F65" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="G65" s="9"/>
+      <c r="G65" s="9" t="s">
+        <v>144</v>
+      </c>
       <c r="H65" s="8">
         <v>12</v>
       </c>
@@ -7679,7 +7684,7 @@
     </row>
     <row r="66" spans="1:27">
       <c r="A66" s="4" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B66" s="5" t="s">
         <v>91</v>
@@ -7760,7 +7765,7 @@
     </row>
     <row r="67" spans="1:27">
       <c r="A67" s="4" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="B67" s="5" t="s">
         <v>91</v>
@@ -7841,7 +7846,7 @@
     </row>
     <row r="68" spans="1:27">
       <c r="A68" s="9" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B68" s="5" t="s">
         <v>91</v>
@@ -7922,7 +7927,7 @@
     </row>
     <row r="69" spans="1:27">
       <c r="A69" s="4" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B69" s="5" t="s">
         <v>91</v>
@@ -8005,7 +8010,7 @@
     </row>
     <row r="70" spans="1:27">
       <c r="A70" s="4" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="B70" s="5" t="s">
         <v>91</v>
@@ -8086,7 +8091,7 @@
     </row>
     <row r="71" spans="1:27">
       <c r="A71" s="20" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B71" s="5" t="s">
         <v>91</v>
@@ -8167,7 +8172,7 @@
     </row>
     <row r="72" spans="1:27">
       <c r="A72" s="12" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B72" s="5" t="s">
         <v>91</v>
@@ -8185,7 +8190,7 @@
         <v>114</v>
       </c>
       <c r="G72" s="7" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="H72" s="8">
         <v>25</v>
@@ -8250,7 +8255,7 @@
     </row>
     <row r="73" spans="1:27">
       <c r="A73" s="4" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B73" s="5" t="s">
         <v>91</v>
@@ -8267,7 +8272,9 @@
       <c r="F73" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="G73" s="9"/>
+      <c r="G73" s="9" t="s">
+        <v>144</v>
+      </c>
       <c r="H73" s="8">
         <v>12</v>
       </c>
@@ -8331,7 +8338,7 @@
     </row>
     <row r="74" spans="1:27">
       <c r="A74" s="5" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B74" s="5" t="s">
         <v>91</v>
@@ -8414,7 +8421,7 @@
     </row>
     <row r="75" spans="1:27">
       <c r="A75" s="4" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B75" s="5" t="s">
         <v>91</v>
@@ -8497,7 +8504,7 @@
     </row>
     <row r="76" spans="1:27">
       <c r="A76" s="4" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="B76" s="5" t="s">
         <v>91</v>
@@ -8578,7 +8585,7 @@
     </row>
     <row r="77" spans="1:27">
       <c r="A77" s="9" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B77" s="5" t="s">
         <v>91</v>
@@ -8659,7 +8666,7 @@
     </row>
     <row r="78" spans="1:27">
       <c r="A78" s="11" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B78" s="5" t="s">
         <v>91</v>
@@ -8677,7 +8684,7 @@
         <v>89</v>
       </c>
       <c r="G78" s="9" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="H78" s="8">
         <v>40</v>
@@ -8742,7 +8749,7 @@
     </row>
     <row r="79" spans="1:27">
       <c r="A79" s="4" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B79" s="5" t="s">
         <v>91</v>
@@ -8825,7 +8832,7 @@
     </row>
     <row r="80" spans="1:27">
       <c r="A80" s="4" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B80" s="5" t="s">
         <v>91</v>
@@ -8906,7 +8913,7 @@
     </row>
     <row r="81" spans="1:27">
       <c r="A81" s="5" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B81" s="5" t="s">
         <v>91</v>
@@ -8989,7 +8996,7 @@
     </row>
     <row r="82" spans="1:27">
       <c r="A82" s="5" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B82" s="5" t="s">
         <v>91</v>
@@ -9007,7 +9014,7 @@
         <v>60</v>
       </c>
       <c r="G82" s="4" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="H82" s="8">
         <v>25</v>
@@ -9072,7 +9079,7 @@
     </row>
     <row r="83" spans="1:27">
       <c r="A83" s="4" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="B83" s="5" t="s">
         <v>91</v>
@@ -9153,7 +9160,7 @@
     </row>
     <row r="84" spans="1:27">
       <c r="A84" s="4" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="B84" s="5" t="s">
         <v>91</v>
@@ -9236,7 +9243,7 @@
     </row>
     <row r="85" spans="1:27">
       <c r="A85" s="17" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B85" s="5" t="s">
         <v>91</v>
@@ -9317,7 +9324,7 @@
     </row>
     <row r="86" spans="1:27">
       <c r="A86" s="12" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="B86" s="5" t="s">
         <v>91</v>
@@ -9398,7 +9405,7 @@
     </row>
     <row r="87" spans="1:27">
       <c r="A87" s="17" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B87" s="5" t="s">
         <v>91</v>
@@ -9479,7 +9486,7 @@
     </row>
     <row r="88" spans="1:27">
       <c r="A88" s="4" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="B88" s="5" t="s">
         <v>91</v>
@@ -9560,7 +9567,7 @@
     </row>
     <row r="89" spans="1:27">
       <c r="A89" s="4" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B89" s="5" t="s">
         <v>91</v>
@@ -9578,7 +9585,7 @@
         <v>89</v>
       </c>
       <c r="G89" s="9" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="H89" s="8">
         <v>30</v>
@@ -9643,7 +9650,7 @@
     </row>
     <row r="90" spans="1:27">
       <c r="A90" s="4" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B90" s="5" t="s">
         <v>91</v>
@@ -9726,7 +9733,7 @@
     </row>
     <row r="91" spans="1:27">
       <c r="A91" s="17" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B91" s="5" t="s">
         <v>91</v>
@@ -9807,7 +9814,7 @@
     </row>
     <row r="92" spans="1:27">
       <c r="A92" s="4" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="B92" s="5" t="s">
         <v>91</v>
@@ -9825,7 +9832,7 @@
         <v>89</v>
       </c>
       <c r="G92" s="9" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H92" s="8">
         <v>35</v>
@@ -9890,7 +9897,7 @@
     </row>
     <row r="93" spans="1:27">
       <c r="A93" s="4" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B93" s="5" t="s">
         <v>91</v>
@@ -9971,7 +9978,7 @@
     </row>
     <row r="94" spans="1:27">
       <c r="A94" s="12" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B94" s="5" t="s">
         <v>91</v>
@@ -10052,7 +10059,7 @@
     </row>
     <row r="95" spans="1:27">
       <c r="A95" s="5" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="B95" s="5" t="s">
         <v>91</v>
@@ -10133,7 +10140,7 @@
     </row>
     <row r="96" spans="1:27">
       <c r="A96" s="5" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B96" s="5" t="s">
         <v>91</v>
@@ -10214,7 +10221,7 @@
     </row>
     <row r="97" spans="1:27">
       <c r="A97" s="5" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="B97" s="5" t="s">
         <v>91</v>
@@ -10232,7 +10239,7 @@
         <v>89</v>
       </c>
       <c r="G97" s="9" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H97" s="8">
         <v>35</v>
@@ -10297,7 +10304,7 @@
     </row>
     <row r="98" spans="1:27">
       <c r="A98" s="4" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B98" s="5" t="s">
         <v>91</v>
@@ -10314,7 +10321,9 @@
       <c r="F98" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="G98" s="9"/>
+      <c r="G98" s="9" t="s">
+        <v>144</v>
+      </c>
       <c r="H98" s="8">
         <v>20</v>
       </c>
@@ -10378,7 +10387,7 @@
     </row>
     <row r="99" spans="1:27">
       <c r="A99" s="4" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B99" s="5" t="s">
         <v>91</v>
@@ -10396,7 +10405,7 @@
         <v>73</v>
       </c>
       <c r="G99" s="9" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="H99" s="8">
         <v>20</v>
@@ -10461,7 +10470,7 @@
     </row>
     <row r="100" spans="1:27">
       <c r="A100" s="11" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="B100" s="5" t="s">
         <v>91</v>
@@ -10479,7 +10488,7 @@
         <v>73</v>
       </c>
       <c r="G100" s="9" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="H100" s="8">
         <v>19</v>
@@ -10544,7 +10553,7 @@
     </row>
     <row r="101" spans="1:27">
       <c r="A101" s="4" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B101" s="5" t="s">
         <v>91</v>
@@ -10625,13 +10634,13 @@
     </row>
     <row r="102" spans="1:27">
       <c r="A102" s="5" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="B102" s="5" t="s">
         <v>91</v>
       </c>
       <c r="C102" s="5" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="D102" s="7" t="s">
         <v>92</v>
@@ -10706,7 +10715,7 @@
     </row>
     <row r="103" spans="1:27">
       <c r="A103" s="4" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="B103" s="5" t="s">
         <v>91</v>
@@ -10724,7 +10733,7 @@
         <v>89</v>
       </c>
       <c r="G103" s="9" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="H103" s="8">
         <v>35</v>
@@ -10789,7 +10798,7 @@
     </row>
     <row r="104" spans="1:27">
       <c r="A104" s="17" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="B104" s="5" t="s">
         <v>91</v>
@@ -10807,7 +10816,7 @@
         <v>89</v>
       </c>
       <c r="G104" s="9" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H104" s="8">
         <v>20</v>
@@ -10872,7 +10881,7 @@
     </row>
     <row r="105" spans="1:27">
       <c r="A105" s="21" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="B105" s="5" t="s">
         <v>91</v>
@@ -10953,7 +10962,7 @@
     </row>
     <row r="106" spans="1:27">
       <c r="A106" s="17" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B106" s="5" t="s">
         <v>91</v>
@@ -10971,7 +10980,7 @@
         <v>89</v>
       </c>
       <c r="G106" s="9" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="H106" s="8">
         <v>16</v>
@@ -11036,7 +11045,7 @@
     </row>
     <row r="107" spans="1:27">
       <c r="A107" s="17" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="B107" s="5" t="s">
         <v>91</v>
@@ -11117,7 +11126,7 @@
     </row>
     <row r="108" spans="1:27">
       <c r="A108" s="18" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="B108" s="5" t="s">
         <v>91</v>
@@ -11198,7 +11207,7 @@
     </row>
     <row r="109" spans="1:27">
       <c r="A109" s="4" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="B109" s="5" t="s">
         <v>91</v>
@@ -11279,7 +11288,7 @@
     </row>
     <row r="110" spans="1:27">
       <c r="A110" s="4" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B110" s="5" t="s">
         <v>91</v>
@@ -11360,7 +11369,7 @@
     </row>
     <row r="111" spans="1:27">
       <c r="A111" s="22" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="B111" s="5" t="s">
         <v>91</v>
@@ -11441,7 +11450,7 @@
     </row>
     <row r="112" spans="1:27">
       <c r="A112" s="23" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B112" s="5" t="s">
         <v>91</v>
@@ -11459,7 +11468,7 @@
         <v>70</v>
       </c>
       <c r="G112" s="4" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="H112" s="8">
         <v>16</v>
@@ -11524,7 +11533,7 @@
     </row>
     <row r="113" spans="1:27">
       <c r="A113" s="4" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="B113" s="5" t="s">
         <v>91</v>
@@ -11605,7 +11614,7 @@
     </row>
     <row r="114" spans="1:27">
       <c r="A114" s="4" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="B114" s="5" t="s">
         <v>91</v>
@@ -11686,7 +11695,7 @@
     </row>
     <row r="115" spans="1:27">
       <c r="A115" s="5" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="B115" s="5" t="s">
         <v>91</v>
@@ -11767,7 +11776,7 @@
     </row>
     <row r="116" spans="1:27">
       <c r="A116" s="4" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B116" s="5" t="s">
         <v>91</v>
@@ -11784,7 +11793,9 @@
       <c r="F116" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="G116" s="9"/>
+      <c r="G116" s="9" t="s">
+        <v>144</v>
+      </c>
       <c r="H116" s="8">
         <v>12</v>
       </c>
@@ -11848,7 +11859,7 @@
     </row>
     <row r="117" spans="1:27">
       <c r="A117" s="4" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="B117" s="5" t="s">
         <v>91</v>
@@ -11866,7 +11877,7 @@
         <v>49</v>
       </c>
       <c r="G117" s="9" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="H117" s="8">
         <v>12</v>
@@ -11931,7 +11942,7 @@
     </row>
     <row r="118" spans="1:27">
       <c r="A118" s="16" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="B118" s="5" t="s">
         <v>91</v>
@@ -12012,7 +12023,7 @@
     </row>
     <row r="119" spans="1:27">
       <c r="A119" s="4" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B119" s="5" t="s">
         <v>91</v>
@@ -12093,7 +12104,7 @@
     </row>
     <row r="120" spans="1:27">
       <c r="A120" s="4" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="B120" s="5" t="s">
         <v>91</v>
@@ -12174,7 +12185,7 @@
     </row>
     <row r="121" spans="1:27">
       <c r="A121" s="4" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="B121" s="5" t="s">
         <v>91</v>
@@ -12257,7 +12268,7 @@
     </row>
     <row r="122" spans="1:27">
       <c r="A122" s="5" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="B122" s="5" t="s">
         <v>91</v>
@@ -12275,7 +12286,7 @@
         <v>89</v>
       </c>
       <c r="G122" s="9" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H122" s="8">
         <v>40</v>
@@ -12340,7 +12351,7 @@
     </row>
     <row r="123" spans="1:27">
       <c r="A123" s="5" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="B123" s="5" t="s">
         <v>91</v>
@@ -12423,7 +12434,7 @@
     </row>
     <row r="124" spans="1:27">
       <c r="A124" s="5" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="B124" s="5" t="s">
         <v>91</v>
@@ -12506,7 +12517,7 @@
     </row>
     <row r="125" spans="1:27">
       <c r="A125" s="4" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="B125" s="5" t="s">
         <v>91</v>
@@ -12587,7 +12598,7 @@
     </row>
     <row r="126" spans="1:27">
       <c r="A126" s="14" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="B126" s="5" t="s">
         <v>91</v>
@@ -12668,7 +12679,7 @@
     </row>
     <row r="127" spans="1:27">
       <c r="A127" s="17" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="B127" s="5" t="s">
         <v>91</v>
@@ -12749,7 +12760,7 @@
     </row>
     <row r="128" spans="1:27">
       <c r="A128" s="5" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="B128" s="5" t="s">
         <v>91</v>
@@ -12830,7 +12841,7 @@
     </row>
     <row r="129" spans="1:27">
       <c r="A129" s="4" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B129" s="5" t="s">
         <v>91</v>
@@ -12911,7 +12922,7 @@
     </row>
     <row r="130" spans="1:27">
       <c r="A130" s="17" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="B130" s="5" t="s">
         <v>91</v>
@@ -12992,7 +13003,7 @@
     </row>
     <row r="131" spans="1:27">
       <c r="A131" s="4" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="B131" s="5" t="s">
         <v>91</v>
@@ -13010,7 +13021,7 @@
         <v>49</v>
       </c>
       <c r="G131" s="9" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="H131" s="8">
         <v>12</v>
@@ -13075,7 +13086,7 @@
     </row>
     <row r="132" spans="1:27">
       <c r="A132" s="11" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="B132" s="5" t="s">
         <v>91</v>
@@ -13156,7 +13167,7 @@
     </row>
     <row r="133" spans="1:27">
       <c r="A133" s="11" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="B133" s="5" t="s">
         <v>91</v>
@@ -13237,7 +13248,7 @@
     </row>
     <row r="134" spans="1:27">
       <c r="A134" s="12" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="B134" s="5" t="s">
         <v>91</v>
@@ -13318,7 +13329,7 @@
     </row>
     <row r="135" spans="1:27">
       <c r="A135" s="4" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="B135" s="5" t="s">
         <v>91</v>
@@ -13399,7 +13410,7 @@
     </row>
     <row r="136" spans="1:27">
       <c r="A136" s="4" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B136" s="5" t="s">
         <v>91</v>
@@ -13417,7 +13428,7 @@
         <v>70</v>
       </c>
       <c r="G136" s="4" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="H136" s="8">
         <v>30</v>
@@ -13482,7 +13493,7 @@
     </row>
     <row r="137" spans="1:27">
       <c r="A137" s="4" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="B137" s="5" t="s">
         <v>91</v>
@@ -13565,7 +13576,7 @@
     </row>
     <row r="138" spans="1:27">
       <c r="A138" s="4" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B138" s="5" t="s">
         <v>29</v>
@@ -13583,7 +13594,7 @@
         <v>84</v>
       </c>
       <c r="G138" s="4" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="H138" s="8">
         <v>220</v>
@@ -13648,7 +13659,7 @@
     </row>
     <row r="139" spans="1:27">
       <c r="A139" s="4" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="B139" s="5" t="s">
         <v>29</v>
@@ -13731,7 +13742,7 @@
     </row>
     <row r="140" spans="1:27">
       <c r="A140" s="4" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B140" s="5" t="s">
         <v>29</v>
@@ -13749,7 +13760,7 @@
         <v>84</v>
       </c>
       <c r="G140" s="9" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="H140" s="8">
         <v>400</v>
@@ -13814,7 +13825,7 @@
     </row>
     <row r="141" spans="1:27">
       <c r="A141" s="4" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="B141" s="5" t="s">
         <v>29</v>
@@ -13895,7 +13906,7 @@
     </row>
     <row r="142" spans="1:27">
       <c r="A142" s="4" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="B142" s="5" t="s">
         <v>29</v>
@@ -13976,7 +13987,7 @@
     </row>
     <row r="143" spans="1:27">
       <c r="A143" s="4" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="B143" s="5" t="s">
         <v>29</v>
@@ -14057,7 +14068,7 @@
     </row>
     <row r="144" spans="1:27">
       <c r="A144" s="24" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="B144" s="5" t="s">
         <v>29</v>
@@ -14140,7 +14151,7 @@
     </row>
     <row r="145" spans="1:28">
       <c r="A145" s="24" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="B145" s="5" t="s">
         <v>29</v>
@@ -14158,7 +14169,7 @@
         <v>60</v>
       </c>
       <c r="G145" s="9" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="H145" s="8">
         <v>45</v>
@@ -14223,7 +14234,7 @@
     </row>
     <row r="146" spans="1:28">
       <c r="A146" s="17" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="B146" s="5" t="s">
         <v>29</v>
@@ -14304,7 +14315,7 @@
     </row>
     <row r="147" spans="1:28">
       <c r="A147" s="4" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="B147" s="5" t="s">
         <v>29</v>
@@ -14390,7 +14401,7 @@
     </row>
     <row r="148" spans="1:28">
       <c r="A148" s="5" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="B148" s="5" t="s">
         <v>29</v>
@@ -14471,7 +14482,7 @@
     </row>
     <row r="149" spans="1:28">
       <c r="A149" s="24" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="B149" s="5" t="s">
         <v>29</v>
@@ -14489,7 +14500,7 @@
         <v>44</v>
       </c>
       <c r="G149" s="4" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="H149" s="8">
         <v>30</v>
@@ -14554,7 +14565,7 @@
     </row>
     <row r="150" spans="1:28">
       <c r="A150" s="24" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B150" s="5" t="s">
         <v>29</v>
@@ -14637,7 +14648,7 @@
     </row>
     <row r="151" spans="1:28">
       <c r="A151" s="24" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="B151" s="5" t="s">
         <v>29</v>
@@ -14723,7 +14734,7 @@
     </row>
     <row r="152" spans="1:28">
       <c r="A152" s="24" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="B152" s="5" t="s">
         <v>29</v>
@@ -14805,7 +14816,7 @@
     </row>
     <row r="153" spans="1:28">
       <c r="A153" s="4" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="B153" s="5" t="s">
         <v>29</v>
@@ -14889,7 +14900,7 @@
     </row>
     <row r="154" spans="1:28">
       <c r="A154" s="11" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="B154" s="5" t="s">
         <v>29</v>
@@ -14971,7 +14982,7 @@
     </row>
     <row r="155" spans="1:28">
       <c r="A155" s="4" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="B155" s="5" t="s">
         <v>29</v>
@@ -15053,7 +15064,7 @@
     </row>
     <row r="156" spans="1:28">
       <c r="A156" s="17" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="B156" s="5" t="s">
         <v>29</v>
@@ -15135,7 +15146,7 @@
     </row>
     <row r="157" spans="1:28">
       <c r="A157" s="4" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="B157" s="5" t="s">
         <v>29</v>
@@ -15219,7 +15230,7 @@
     </row>
     <row r="158" spans="1:28">
       <c r="A158" s="4" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="B158" s="5" t="s">
         <v>29</v>
@@ -15237,7 +15248,7 @@
         <v>41</v>
       </c>
       <c r="G158" s="4" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="H158" s="8">
         <v>130</v>
@@ -15303,7 +15314,7 @@
     </row>
     <row r="159" spans="1:28">
       <c r="A159" s="17" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="B159" s="5" t="s">
         <v>29</v>
@@ -15385,7 +15396,7 @@
     </row>
     <row r="160" spans="1:28">
       <c r="A160" s="4" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="B160" s="5" t="s">
         <v>29</v>
@@ -15467,7 +15478,7 @@
     </row>
     <row r="161" spans="1:28">
       <c r="A161" s="4" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="B161" s="5" t="s">
         <v>29</v>
@@ -15549,7 +15560,7 @@
     </row>
     <row r="162" spans="1:28">
       <c r="A162" s="4" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="B162" s="5" t="s">
         <v>29</v>
@@ -15566,7 +15577,9 @@
       <c r="F162" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="G162" s="9"/>
+      <c r="G162" s="9" t="s">
+        <v>144</v>
+      </c>
       <c r="H162" s="8">
         <v>20</v>
       </c>
@@ -15633,7 +15646,7 @@
     </row>
     <row r="163" spans="1:28">
       <c r="A163" s="4" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="B163" s="5" t="s">
         <v>29</v>
@@ -15651,7 +15664,7 @@
         <v>60</v>
       </c>
       <c r="G163" s="4" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="H163" s="8">
         <v>185</v>
@@ -15717,7 +15730,7 @@
     </row>
     <row r="164" spans="1:28">
       <c r="A164" s="17" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="B164" s="5" t="s">
         <v>29</v>
@@ -15735,7 +15748,7 @@
         <v>84</v>
       </c>
       <c r="G164" s="25" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="H164" s="8">
         <v>60</v>
@@ -15801,7 +15814,7 @@
     </row>
     <row r="165" spans="1:28">
       <c r="A165" s="4" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="B165" s="5" t="s">
         <v>29</v>
@@ -15883,7 +15896,7 @@
     </row>
     <row r="166" spans="1:28">
       <c r="A166" s="4" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="B166" s="5" t="s">
         <v>29</v>
@@ -15901,7 +15914,7 @@
         <v>84</v>
       </c>
       <c r="G166" s="4" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="H166" s="8">
         <v>150</v>
@@ -15967,7 +15980,7 @@
     </row>
     <row r="167" spans="1:28">
       <c r="A167" s="4" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="B167" s="5" t="s">
         <v>29</v>
@@ -15985,7 +15998,7 @@
         <v>84</v>
       </c>
       <c r="G167" s="4" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="H167" s="8">
         <v>65</v>
@@ -16051,7 +16064,7 @@
     </row>
     <row r="168" spans="1:28">
       <c r="A168" s="4" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="B168" s="5" t="s">
         <v>29</v>
@@ -16137,7 +16150,7 @@
     </row>
     <row r="169" spans="1:28">
       <c r="A169" s="17" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="B169" s="5" t="s">
         <v>29</v>
@@ -16219,7 +16232,7 @@
     </row>
     <row r="170" spans="1:28">
       <c r="A170" s="17" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="B170" s="5" t="s">
         <v>29</v>
@@ -16237,7 +16250,7 @@
         <v>70</v>
       </c>
       <c r="G170" s="4" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="H170" s="8">
         <v>25</v>
@@ -16303,7 +16316,7 @@
     </row>
     <row r="171" spans="1:28">
       <c r="A171" s="17" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="B171" s="5" t="s">
         <v>29</v>
@@ -16385,7 +16398,7 @@
     </row>
     <row r="172" spans="1:28">
       <c r="A172" s="17" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="B172" s="5" t="s">
         <v>29</v>
@@ -16469,7 +16482,7 @@
     </row>
     <row r="173" spans="1:28">
       <c r="A173" s="4" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="B173" s="5" t="s">
         <v>29</v>
@@ -16487,7 +16500,7 @@
         <v>41</v>
       </c>
       <c r="G173" s="4" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="H173" s="8">
         <v>220</v>
@@ -16553,7 +16566,7 @@
     </row>
     <row r="174" spans="1:28">
       <c r="A174" s="4" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="B174" s="5" t="s">
         <v>29</v>
@@ -16637,7 +16650,7 @@
     </row>
     <row r="175" spans="1:28">
       <c r="A175" s="4" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="B175" s="5" t="s">
         <v>29</v>
@@ -16655,7 +16668,7 @@
         <v>49</v>
       </c>
       <c r="G175" s="9" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="H175" s="8">
         <v>20</v>
@@ -16723,7 +16736,7 @@
     </row>
     <row r="176" spans="1:28">
       <c r="A176" s="4" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="B176" s="5" t="s">
         <v>29</v>
@@ -16741,7 +16754,7 @@
         <v>73</v>
       </c>
       <c r="G176" s="9" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="H176" s="8">
         <v>30</v>
@@ -16807,7 +16820,7 @@
     </row>
     <row r="177" spans="1:28">
       <c r="A177" s="4" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="B177" s="5" t="s">
         <v>29</v>
@@ -16825,7 +16838,7 @@
         <v>44</v>
       </c>
       <c r="G177" s="4" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="H177" s="8">
         <v>240</v>
@@ -16891,13 +16904,13 @@
     </row>
     <row r="178" spans="1:28">
       <c r="A178" s="4" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="B178" s="5" t="s">
         <v>91</v>
       </c>
       <c r="C178" s="5" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="D178" s="7" t="s">
         <v>111</v>
@@ -16973,13 +16986,13 @@
     </row>
     <row r="179" spans="1:28">
       <c r="A179" s="4" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="B179" s="5" t="s">
         <v>91</v>
       </c>
       <c r="C179" s="5" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="D179" s="7" t="s">
         <v>96</v>
@@ -17055,13 +17068,13 @@
     </row>
     <row r="180" spans="1:28">
       <c r="A180" s="4" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="B180" s="5" t="s">
         <v>91</v>
       </c>
       <c r="C180" s="5" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="D180" s="7" t="s">
         <v>96</v>
@@ -17137,13 +17150,13 @@
     </row>
     <row r="181" spans="1:28">
       <c r="A181" s="4" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="B181" s="5" t="s">
         <v>91</v>
       </c>
       <c r="C181" s="5" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="D181" s="7" t="s">
         <v>111</v>
@@ -17219,13 +17232,13 @@
     </row>
     <row r="182" spans="1:28">
       <c r="A182" s="4" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="B182" s="5" t="s">
         <v>91</v>
       </c>
       <c r="C182" s="5" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="D182" s="7" t="s">
         <v>111</v>
@@ -17301,13 +17314,13 @@
     </row>
     <row r="183" spans="1:28">
       <c r="A183" s="4" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="B183" s="5" t="s">
         <v>91</v>
       </c>
       <c r="C183" s="5" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="D183" s="6" t="s">
         <v>122</v>
@@ -17383,7 +17396,7 @@
     </row>
     <row r="184" spans="1:28">
       <c r="A184" s="4" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="B184" s="5" t="s">
         <v>29</v>
@@ -17465,7 +17478,7 @@
     </row>
     <row r="185" spans="1:28">
       <c r="A185" s="4" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="B185" s="5" t="s">
         <v>29</v>
@@ -17547,7 +17560,7 @@
     </row>
     <row r="186" spans="1:28">
       <c r="A186" s="4" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="B186" s="5" t="s">
         <v>29</v>
@@ -17565,7 +17578,7 @@
         <v>41</v>
       </c>
       <c r="G186" s="4" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="H186" s="8">
         <v>250</v>
@@ -17631,7 +17644,7 @@
     </row>
     <row r="187" spans="1:28">
       <c r="A187" s="4" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="B187" s="5" t="s">
         <v>29</v>
@@ -17715,7 +17728,7 @@
     </row>
     <row r="188" spans="1:28">
       <c r="A188" s="4" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="B188" s="5" t="s">
         <v>29</v>
@@ -17733,7 +17746,7 @@
         <v>41</v>
       </c>
       <c r="G188" s="4" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="H188" s="8">
         <v>390</v>
@@ -17799,7 +17812,7 @@
     </row>
     <row r="189" spans="1:28">
       <c r="A189" s="4" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="B189" s="5" t="s">
         <v>29</v>
@@ -17881,7 +17894,7 @@
     </row>
     <row r="190" spans="1:28">
       <c r="A190" s="26" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="B190" s="5" t="s">
         <v>29</v>
@@ -17963,7 +17976,7 @@
     </row>
     <row r="191" spans="1:28">
       <c r="A191" s="17" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="B191" s="5" t="s">
         <v>29</v>
@@ -18045,7 +18058,7 @@
     </row>
     <row r="192" spans="1:28">
       <c r="A192" s="4" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="B192" s="5" t="s">
         <v>29</v>
@@ -18129,7 +18142,7 @@
     </row>
     <row r="193" spans="1:28">
       <c r="A193" s="4" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="B193" s="5" t="s">
         <v>29</v>
@@ -18211,7 +18224,7 @@
     </row>
     <row r="194" spans="1:28">
       <c r="A194" s="4" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="B194" s="5" t="s">
         <v>29</v>
@@ -18293,7 +18306,7 @@
     </row>
     <row r="195" spans="1:28">
       <c r="A195" s="17" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="B195" s="5" t="s">
         <v>29</v>
@@ -18377,13 +18390,13 @@
     </row>
     <row r="196" spans="1:28">
       <c r="A196" s="17" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="B196" s="5" t="s">
         <v>91</v>
       </c>
       <c r="C196" s="5" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="D196" s="6" t="s">
         <v>100</v>
@@ -18459,13 +18472,13 @@
     </row>
     <row r="197" spans="1:28">
       <c r="A197" s="4" t="s">
+        <v>292</v>
+      </c>
+      <c r="B197" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="C197" s="5" t="s">
         <v>291</v>
-      </c>
-      <c r="B197" s="5" t="s">
-        <v>91</v>
-      </c>
-      <c r="C197" s="5" t="s">
-        <v>290</v>
       </c>
       <c r="D197" s="6" t="s">
         <v>100</v>
@@ -18541,13 +18554,13 @@
     </row>
     <row r="198" spans="1:28">
       <c r="A198" s="24" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="B198" s="5" t="s">
         <v>91</v>
       </c>
       <c r="C198" s="5" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="D198" s="7" t="s">
         <v>94</v>
@@ -18623,7 +18636,7 @@
     </row>
     <row r="199" spans="1:28">
       <c r="A199" s="24" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="B199" s="5" t="s">
         <v>91</v>
@@ -18707,13 +18720,13 @@
     </row>
     <row r="200" spans="1:28">
       <c r="A200" s="24" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="B200" s="5" t="s">
         <v>91</v>
       </c>
       <c r="C200" s="5" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="D200" s="7" t="s">
         <v>94</v>
@@ -18789,13 +18802,13 @@
     </row>
     <row r="201" spans="1:28">
       <c r="A201" s="24" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="B201" s="5" t="s">
         <v>91</v>
       </c>
       <c r="C201" s="5" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="D201" s="7" t="s">
         <v>111</v>
@@ -18871,13 +18884,13 @@
     </row>
     <row r="202" spans="1:28">
       <c r="A202" s="20" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="B202" s="5" t="s">
         <v>91</v>
       </c>
       <c r="C202" s="5" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="D202" s="6" t="s">
         <v>109</v>
@@ -18953,13 +18966,13 @@
     </row>
     <row r="203" spans="1:28">
       <c r="A203" s="17" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="B203" s="5" t="s">
         <v>91</v>
       </c>
       <c r="C203" s="5" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="D203" s="7" t="s">
         <v>107</v>
@@ -19035,13 +19048,13 @@
     </row>
     <row r="204" spans="1:28">
       <c r="A204" s="4" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="B204" s="5" t="s">
         <v>91</v>
       </c>
       <c r="C204" s="5" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="D204" s="7" t="s">
         <v>92</v>
@@ -19117,13 +19130,13 @@
     </row>
     <row r="205" spans="1:28">
       <c r="A205" s="4" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="B205" s="5" t="s">
         <v>91</v>
       </c>
       <c r="C205" s="5" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="D205" s="6" t="s">
         <v>122</v>
@@ -19199,13 +19212,13 @@
     </row>
     <row r="206" spans="1:28">
       <c r="A206" s="4" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="B206" s="5" t="s">
         <v>91</v>
       </c>
       <c r="C206" s="5" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="D206" s="7" t="s">
         <v>96</v>
@@ -19281,13 +19294,13 @@
     </row>
     <row r="207" spans="1:28">
       <c r="A207" s="4" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="B207" s="5" t="s">
         <v>91</v>
       </c>
       <c r="C207" s="5" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="D207" s="7" t="s">
         <v>96</v>
@@ -19363,13 +19376,13 @@
     </row>
     <row r="208" spans="1:28">
       <c r="A208" s="4" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="B208" s="5" t="s">
         <v>91</v>
       </c>
       <c r="C208" s="5" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="D208" s="7" t="s">
         <v>107</v>
@@ -19445,13 +19458,13 @@
     </row>
     <row r="209" spans="1:28">
       <c r="A209" s="4" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="B209" s="5" t="s">
         <v>91</v>
       </c>
       <c r="C209" s="5" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="D209" s="7" t="s">
         <v>94</v>
@@ -19527,13 +19540,13 @@
     </row>
     <row r="210" spans="1:28">
       <c r="A210" s="4" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="B210" s="5" t="s">
         <v>91</v>
       </c>
       <c r="C210" s="5" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="D210" s="7" t="s">
         <v>96</v>
@@ -19609,13 +19622,13 @@
     </row>
     <row r="211" spans="1:28">
       <c r="A211" s="4" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="B211" s="5" t="s">
         <v>91</v>
       </c>
       <c r="C211" s="5" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="D211" s="7" t="s">
         <v>111</v>
@@ -19691,13 +19704,13 @@
     </row>
     <row r="212" spans="1:28">
       <c r="A212" s="4" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="B212" s="5" t="s">
         <v>91</v>
       </c>
       <c r="C212" s="5" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="D212" s="7" t="s">
         <v>96</v>
@@ -19773,13 +19786,13 @@
     </row>
     <row r="213" spans="1:28">
       <c r="A213" s="4" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="B213" s="5" t="s">
         <v>91</v>
       </c>
       <c r="C213" s="5" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="D213" s="7" t="s">
         <v>92</v>
@@ -19855,7 +19868,7 @@
     </row>
     <row r="214" spans="1:28">
       <c r="A214" s="17" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="B214" s="5" t="s">
         <v>29</v>
@@ -19873,7 +19886,7 @@
         <v>49</v>
       </c>
       <c r="G214" s="9" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="H214" s="8">
         <v>12</v>
@@ -19941,7 +19954,7 @@
     </row>
     <row r="215" spans="1:28">
       <c r="A215" s="24" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="B215" s="5" t="s">
         <v>29</v>
@@ -20023,7 +20036,7 @@
     </row>
     <row r="216" spans="1:28">
       <c r="A216" s="4" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="B216" s="5" t="s">
         <v>29</v>
@@ -20107,7 +20120,7 @@
     </row>
     <row r="217" spans="1:28">
       <c r="A217" s="4" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="B217" s="5" t="s">
         <v>29</v>
@@ -20189,7 +20202,7 @@
     </row>
     <row r="218" spans="1:28">
       <c r="A218" s="24" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="B218" s="5" t="s">
         <v>29</v>
@@ -20273,7 +20286,7 @@
     </row>
     <row r="219" spans="1:28">
       <c r="A219" s="4" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="B219" s="5" t="s">
         <v>29</v>
@@ -20355,7 +20368,7 @@
     </row>
     <row r="220" spans="1:28">
       <c r="A220" s="29" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="B220" s="5" t="s">
         <v>29</v>
@@ -20437,7 +20450,7 @@
     </row>
     <row r="221" spans="1:28">
       <c r="A221" s="5" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="B221" s="5" t="s">
         <v>29</v>
@@ -20521,7 +20534,7 @@
     </row>
     <row r="222" spans="1:28">
       <c r="A222" s="5" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="B222" s="5" t="s">
         <v>29</v>
@@ -20603,7 +20616,7 @@
     </row>
     <row r="223" spans="1:28">
       <c r="A223" s="4" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="B223" s="5" t="s">
         <v>29</v>
@@ -20621,7 +20634,7 @@
         <v>32</v>
       </c>
       <c r="G223" s="9" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="H223" s="8">
         <v>35</v>
@@ -20687,7 +20700,7 @@
     </row>
     <row r="224" spans="1:28">
       <c r="A224" s="4" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="B224" s="5" t="s">
         <v>29</v>
@@ -20769,7 +20782,7 @@
     </row>
     <row r="225" spans="1:28">
       <c r="A225" s="4" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="B225" s="5" t="s">
         <v>29</v>
@@ -20853,7 +20866,7 @@
     </row>
     <row r="226" spans="1:28">
       <c r="A226" s="4" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="B226" s="5" t="s">
         <v>29</v>
@@ -20937,7 +20950,7 @@
     </row>
     <row r="227" spans="1:28">
       <c r="A227" s="4" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="B227" s="5" t="s">
         <v>29</v>
@@ -20955,7 +20968,7 @@
         <v>84</v>
       </c>
       <c r="G227" s="4" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="H227" s="8">
         <v>60</v>
@@ -21021,7 +21034,7 @@
     </row>
     <row r="228" spans="1:28">
       <c r="A228" s="4" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="B228" s="5" t="s">
         <v>29</v>
@@ -21039,7 +21052,7 @@
         <v>32</v>
       </c>
       <c r="G228" s="7" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="H228" s="8">
         <v>300</v>
@@ -21105,7 +21118,7 @@
     </row>
     <row r="229" spans="1:28">
       <c r="A229" s="11" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="B229" s="5" t="s">
         <v>29</v>
@@ -21187,7 +21200,7 @@
     </row>
     <row r="230" spans="1:28">
       <c r="A230" s="4" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="B230" s="5" t="s">
         <v>29</v>
@@ -21205,7 +21218,7 @@
         <v>44</v>
       </c>
       <c r="G230" s="4" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="H230" s="8">
         <v>30</v>
@@ -21271,7 +21284,7 @@
     </row>
     <row r="231" spans="1:28">
       <c r="A231" s="4" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="B231" s="5" t="s">
         <v>29</v>
@@ -21289,7 +21302,7 @@
         <v>114</v>
       </c>
       <c r="G231" s="7" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="H231" s="8">
         <v>90</v>
@@ -21355,7 +21368,7 @@
     </row>
     <row r="232" spans="1:28">
       <c r="A232" s="4" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="B232" s="5" t="s">
         <v>29</v>
@@ -21439,7 +21452,7 @@
     </row>
     <row r="233" spans="1:28">
       <c r="A233" s="4" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="B233" s="5" t="s">
         <v>29</v>
@@ -21523,7 +21536,7 @@
     </row>
     <row r="234" spans="1:28">
       <c r="A234" s="4" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="B234" s="5" t="s">
         <v>29</v>
@@ -21541,7 +21554,7 @@
         <v>44</v>
       </c>
       <c r="G234" s="4" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="H234" s="8">
         <v>220</v>
@@ -21607,7 +21620,7 @@
     </row>
     <row r="235" spans="1:28">
       <c r="A235" s="4" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="B235" s="5" t="s">
         <v>29</v>
@@ -21625,7 +21638,7 @@
         <v>70</v>
       </c>
       <c r="G235" s="4" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="H235" s="8">
         <v>232</v>
@@ -21691,7 +21704,7 @@
     </row>
     <row r="236" spans="1:28">
       <c r="A236" s="4" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="B236" s="5" t="s">
         <v>29</v>
@@ -21775,7 +21788,7 @@
     </row>
     <row r="237" spans="1:28">
       <c r="A237" s="4" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="B237" s="5" t="s">
         <v>29</v>

</xml_diff>